<commit_message>
chore: add test data, config modules, and helpers; remove form.html
</commit_message>
<xml_diff>
--- a/Data Input Pengujian/LPH 2026/6. LPH JUNI/Lap. Produksi Harian 2026-06-02 - 2026-06-02.xlsx
+++ b/Data Input Pengujian/LPH 2026/6. LPH JUNI/Lap. Produksi Harian 2026-06-02 - 2026-06-02.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Python\odooCompressionTest\Data Input Pengujian\LPH 2026\6. LPH JUNI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9358536B-04A3-4FB9-8095-6CDDBADB3772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A017296-C47F-4261-9E51-77C3C02F155A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1115,32 +1115,32 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" t="s">
+    <row r="12" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C12" t="s">
-        <v>121</v>
-      </c>
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" t="s">
-        <v>122</v>
-      </c>
-      <c r="F12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="C12" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12" s="2" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1260,32 +1260,32 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>9</v>
-      </c>
-      <c r="B17" t="s">
+    <row r="17" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C17" t="s">
-        <v>121</v>
-      </c>
-      <c r="D17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" t="s">
-        <v>122</v>
-      </c>
-      <c r="F17" t="s">
-        <v>12</v>
-      </c>
-      <c r="G17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H17" t="s">
+      <c r="C17" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I17" t="s">
+      <c r="I17" s="2" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1521,32 +1521,32 @@
         <v>65</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>9</v>
-      </c>
-      <c r="B26" t="s">
+    <row r="26" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C26" t="s">
-        <v>121</v>
-      </c>
-      <c r="D26" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" t="s">
-        <v>122</v>
-      </c>
-      <c r="F26" t="s">
-        <v>12</v>
-      </c>
-      <c r="G26" t="s">
-        <v>13</v>
-      </c>
-      <c r="H26" t="s">
+      <c r="C26" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="I26" t="s">
+      <c r="I26" s="2" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1695,32 +1695,32 @@
         <v>39</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>9</v>
-      </c>
-      <c r="B32" t="s">
+    <row r="32" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C32" t="s">
-        <v>121</v>
-      </c>
-      <c r="D32" t="s">
-        <v>11</v>
-      </c>
-      <c r="E32" t="s">
-        <v>122</v>
-      </c>
-      <c r="F32" t="s">
-        <v>12</v>
-      </c>
-      <c r="G32" t="s">
-        <v>13</v>
-      </c>
-      <c r="H32" t="s">
+      <c r="C32" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H32" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="I32" t="s">
+      <c r="I32" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1811,32 +1811,32 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>9</v>
-      </c>
-      <c r="B36" t="s">
+    <row r="36" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C36" t="s">
-        <v>121</v>
-      </c>
-      <c r="D36" t="s">
-        <v>11</v>
-      </c>
-      <c r="E36" t="s">
-        <v>122</v>
-      </c>
-      <c r="F36" t="s">
-        <v>12</v>
-      </c>
-      <c r="G36" t="s">
-        <v>13</v>
-      </c>
-      <c r="H36" t="s">
+      <c r="C36" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H36" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I36" t="s">
+      <c r="I36" s="2" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1898,32 +1898,32 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>9</v>
-      </c>
-      <c r="B39" t="s">
+    <row r="39" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E39" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F39" t="s">
+      <c r="F39" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G39" t="s">
+      <c r="G39" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="H39" t="s">
+      <c r="H39" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="I39" t="s">
+      <c r="I39" s="2" t="s">
         <v>74</v>
       </c>
     </row>
@@ -2014,32 +2014,32 @@
         <v>80</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>9</v>
-      </c>
-      <c r="B43" t="s">
+    <row r="43" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="D43" t="s">
+      <c r="D43" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E43" t="s">
+      <c r="E43" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F43" t="s">
+      <c r="F43" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G43" t="s">
+      <c r="G43" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="H43" t="s">
+      <c r="H43" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="I43" t="s">
+      <c r="I43" s="2" t="s">
         <v>82</v>
       </c>
     </row>
@@ -2101,32 +2101,32 @@
         <v>86</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>9</v>
-      </c>
-      <c r="B46" t="s">
+    <row r="46" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D46" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E46" t="s">
+      <c r="E46" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F46" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G46" t="s">
+      <c r="G46" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="H46" t="s">
+      <c r="H46" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="I46" t="s">
+      <c r="I46" s="2" t="s">
         <v>88</v>
       </c>
     </row>

</xml_diff>